<commit_message>
Correccion de errores en evaluacion rapida y relacion semantica
</commit_message>
<xml_diff>
--- a/data/redneet_db/rib.xlsx
+++ b/data/redneet_db/rib.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnvelasco/Documents/APPs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnvelasco/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F41F8D3-6033-504F-AA54-F18D7BD15760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684F965C-EF78-514D-8998-44ED34CCB4AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16600" xr2:uid="{70B45474-F9F8-1B4B-ABEB-2F870154A49C}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{70B45474-F9F8-1B4B-ABEB-2F870154A49C}"/>
   </bookViews>
   <sheets>
     <sheet name="INDICADORES" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -563,7 +563,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5">
-        <v>3.0394046561442289</v>
+        <v>9.3370818963890851</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -571,7 +571,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6">
-        <v>0.59950932982509675</v>
+        <v>0.31892462330003668</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -579,7 +579,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="5">
-        <v>69.866484432288942</v>
+        <v>69.228880069475423</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -587,7 +587,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="7">
-        <v>0.60904560152343734</v>
+        <v>0.22003094550681487</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -595,7 +595,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5">
-        <v>0.2439170811211985</v>
+        <v>0.14985765909670304</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -603,7 +603,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="8">
-        <v>5744148157</v>
+        <v>4317675061</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -611,7 +611,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="9">
-        <v>3507307935</v>
+        <v>3418615201</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -619,7 +619,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="10">
-        <v>8560729035</v>
+        <v>4835563108</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -627,7 +627,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="10">
-        <v>8757527194</v>
+        <v>5019437375</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -635,7 +635,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="10">
-        <v>2816580878</v>
+        <v>517888047</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -643,7 +643,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="10">
-        <v>5250219259</v>
+        <v>1600822174</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -651,7 +651,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="10">
-        <v>3507307935</v>
+        <v>3418615201</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -659,7 +659,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="10">
-        <v>2136110471</v>
+        <v>752201135</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -667,7 +667,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="10">
-        <v>30574180</v>
+        <v>10865424</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.2">
@@ -675,7 +675,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="11">
-        <v>1318616529.25</v>
+        <v>389535688.25</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.2">
@@ -683,7 +683,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="11">
-        <v>12071423.416666666</v>
+        <v>28072777.333333332</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -691,7 +691,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="11">
-        <v>1330687952.6666667</v>
+        <v>417608465.58333331</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -699,7 +699,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="11">
-        <v>1146556765.0833333</v>
+        <v>333812290.83333331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>